<commit_message>
chore: regenerate manifest xlsx workbooks
</commit_message>
<xml_diff>
--- a/excel_templates/immunopeptidomics_manifest_template.xlsx
+++ b/excel_templates/immunopeptidomics_manifest_template.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Lists" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data Dictionary'!$A$1:$G$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data Dictionary'!$A$1:$G$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>"FASTQ", "BAM", "BAI", "CRAM", "CRAI", "GVCF", "VCF", "TBI", "MAF", "PDF", "HTML", "DCM", "IDAT", "SVS", "GPR", "CNS", "TXT", "PNG", "CSV", "PED", "SEG", "TAR", "TSV", "mzML", "raw"</t>
+          <t>"FASTQ", "BAM", "BAI", "CRAM", "CRAI", "GVCF", "VCF", "TBI", "MAF", "PDF", "HTML", "DCM", "IDAT", "SVS", "GPR", "CNS", "TXT", "PNG", "CSV", "PED", "SEG", "TAR", "TSV", "MZML", "RAW"</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>RAW</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
@@ -1750,7 +1750,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>PI_name</t>
+          <t>FFPE</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -1760,30 +1760,30 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Principal Investigator of the project</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr"/>
+          <t>Is the sample preserved in FFPE</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>"True", "False"</t>
+        </is>
+      </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Fonseca</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>project</t>
+          <t>PI_name</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>Short name of the project</t>
+          <t>Principal Investigator of the project</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr"/>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>RBT</t>
+          <t>Fonseca</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -1816,7 +1816,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>organism</t>
+          <t>project</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -1826,14 +1826,10 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Binomial name of organism with full genus name</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>"Homo sapiens", "Mus musculus"</t>
-        </is>
-      </c>
+          <t>Short name of the project</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr">
         <is>
           <t>string</t>
@@ -1841,30 +1837,34 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Homo sapiens</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr"/>
+          <t>RBT</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>host_organism</t>
+          <t>organism</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Host organism binomial name when the sequenced sample is a xenograft. Required when compisition is "Patient Derived Xenograft" or "Xenograft"</t>
+          <t>Binomial name of organism with full genus name</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>"Mus musculus"</t>
+          <t>"Homo sapiens", "Mus musculus"</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -1874,50 +1874,83 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Mus musculus</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
+          <t>Homo sapiens</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>host_organism</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>Host organism binomial name when the sequenced sample is a xenograft. Required when compisition is "Patient Derived Xenograft" or "Xenograft"</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>"Mus musculus"</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Mus musculus</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
           <t>reported_gender</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>False</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Reported gender of the participant. Required when organism is "Homo sapiens"</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>"Female", "Male", "Not Reported"</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="G48" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G48"/>
+  <autoFilter ref="A1:G49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1928,7 +1961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU1"/>
+  <dimension ref="A1:AV1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1978,6 +2011,7 @@
     <col width="24" customWidth="1" min="45" max="45"/>
     <col width="24" customWidth="1" min="46" max="46"/>
     <col width="24" customWidth="1" min="47" max="47"/>
+    <col width="24" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2193,32 +2227,37 @@
       </c>
       <c r="AQ1" s="1" t="inlineStr">
         <is>
+          <t>FFPE</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
           <t>PI_name</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>project</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>organism</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>host_organism</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>reported_gender</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="14">
+  <dataValidations count="15">
     <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Lists'!$A$2:$A$6</formula1>
     </dataValidation>
@@ -2252,14 +2291,17 @@
     <dataValidation sqref="AO2:AO1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Lists'!$K$2:$K$3</formula1>
     </dataValidation>
-    <dataValidation sqref="AS2:AS1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AQ2:AQ1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Lists'!$L$2:$L$3</formula1>
     </dataValidation>
     <dataValidation sqref="AT2:AT1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Lists'!$M$2:$M$2</formula1>
+      <formula1>'Lists'!$M$2:$M$3</formula1>
     </dataValidation>
     <dataValidation sqref="AU2:AU1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Lists'!$N$2:$N$4</formula1>
+      <formula1>'Lists'!$N$2:$N$2</formula1>
+    </dataValidation>
+    <dataValidation sqref="AV2:AV1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'Lists'!$O$2:$O$4</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2272,7 +2314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2333,15 +2375,20 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>FFPE</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>organism</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>host_organism</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>reported_gender</t>
         </is>
@@ -2405,15 +2452,20 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>Homo sapiens</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Mus musculus</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Female</t>
         </is>
@@ -2472,10 +2524,15 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>Mus musculus</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Male</t>
         </is>
@@ -2512,7 +2569,7 @@
           <t>SHA256</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Not Reported</t>
         </is>
@@ -2831,14 +2888,14 @@
     <row r="25">
       <c r="E25" t="inlineStr">
         <is>
-          <t>mzML</t>
+          <t>MZML</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="E26" t="inlineStr">
         <is>
-          <t>raw</t>
+          <t>RAW</t>
         </is>
       </c>
     </row>

</xml_diff>